<commit_message>
build: 更新 ItemGroupTable 和 TreasureBoxTable 配置
同步数据表配置的最新调整。
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/TreasureBoxTable.xlsx
+++ b/AAAGameData/DataTables/TreasureBoxTable.xlsx
@@ -1210,10 +1210,10 @@
         <v>0</v>
       </c>
       <c r="F5" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H5" s="2">
         <v>1</v>

</xml_diff>